<commit_message>
Update data file: KIOSC_Finance_Data.xlsx
</commit_message>
<xml_diff>
--- a/data/KIOSC_Finance_Data.xlsx
+++ b/data/KIOSC_Finance_Data.xlsx
@@ -462,7 +462,7 @@
       <c r="D2" t="str">
         <v>38d55a28-9ed7-4fab-b86e-cca27fce1cdb</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="str">
         <v>5699.99</v>
       </c>
       <c r="F2" t="str">
@@ -506,7 +506,7 @@
       <c r="D3" t="str">
         <v>11139606-2bf4-4e27-a5e6-581233416593</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="str">
         <v>824.5</v>
       </c>
       <c r="F3" t="str">
@@ -550,7 +550,7 @@
       <c r="D4" t="str">
         <v>f99c571b-2d0d-48a8-b6fa-ec0a2bc491c9</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="str">
         <v>3450</v>
       </c>
       <c r="F4" t="str">
@@ -570,6 +570,9 @@
       </c>
       <c r="K4" t="str">
         <v>2023-02-20</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
       </c>
       <c r="M4" t="str">
         <v>user</v>
@@ -591,7 +594,7 @@
       <c r="D5" t="str">
         <v>f70c0036-d2f2-49f2-b82b-9e25b4857a76</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="str">
         <v>2750</v>
       </c>
       <c r="F5" t="str">
@@ -608,6 +611,12 @@
       </c>
       <c r="J5" t="str">
         <v>Leadership training for department heads</v>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
       </c>
       <c r="M5" t="str">
         <v>admin</v>
@@ -629,7 +638,7 @@
       <c r="D6" t="str">
         <v>2bdb9f5a-ad0a-4722-9bbd-1568a4d448c8</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="str">
         <v>1200</v>
       </c>
       <c r="F6" t="str">
@@ -673,7 +682,7 @@
       <c r="D7" t="str">
         <v>38d55a28-9ed7-4fab-b86e-cca27fce1cdb</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="str">
         <v>3599</v>
       </c>
       <c r="F7" t="str">
@@ -987,7 +996,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" t="str">
         <v>1</v>
       </c>
       <c r="B2" t="str">
@@ -996,12 +1005,12 @@
       <c r="C2" t="str">
         <v>Day-to-day operational expenses</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="str">
         <v>250000</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
+      <c r="A3" t="str">
         <v>2</v>
       </c>
       <c r="B3" t="str">
@@ -1010,12 +1019,12 @@
       <c r="C3" t="str">
         <v>Community outreach and education</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="str">
         <v>75000</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
+      <c r="A4" t="str">
         <v>3</v>
       </c>
       <c r="B4" t="str">
@@ -1024,12 +1033,12 @@
       <c r="C4" t="str">
         <v>Research and development projects</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="str">
         <v>120000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5">
+      <c r="A5" t="str">
         <v>4</v>
       </c>
       <c r="B5" t="str">
@@ -1038,12 +1047,12 @@
       <c r="C5" t="str">
         <v>Infrastructure maintenance and upgrades</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="str">
         <v>180000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6">
+      <c r="A6" t="str">
         <v>5</v>
       </c>
       <c r="B6" t="str">
@@ -1052,7 +1061,7 @@
       <c r="C6" t="str">
         <v>Training and professional development</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="str">
         <v>50000</v>
       </c>
     </row>
@@ -1079,7 +1088,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" t="str">
         <v>1</v>
       </c>
       <c r="B2" t="str">
@@ -1090,7 +1099,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
+      <c r="A3" t="str">
         <v>2</v>
       </c>
       <c r="B3" t="str">
@@ -1101,7 +1110,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4">
+      <c r="A4" t="str">
         <v>3</v>
       </c>
       <c r="B4" t="str">
@@ -1112,7 +1121,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5">
+      <c r="A5" t="str">
         <v>4</v>
       </c>
       <c r="B5" t="str">
@@ -1145,7 +1154,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" t="str">
         <v>1</v>
       </c>
       <c r="B2" t="str">
@@ -1156,7 +1165,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
+      <c r="A3" t="str">
         <v>2</v>
       </c>
       <c r="B3" t="str">
@@ -1167,7 +1176,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4">
+      <c r="A4" t="str">
         <v>3</v>
       </c>
       <c r="B4" t="str">
@@ -1200,7 +1209,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" t="str">
         <v>1</v>
       </c>
       <c r="B2" t="str">
@@ -1211,7 +1220,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
+      <c r="A3" t="str">
         <v>2</v>
       </c>
       <c r="B3" t="str">
@@ -1222,7 +1231,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4">
+      <c r="A4" t="str">
         <v>3</v>
       </c>
       <c r="B4" t="str">
@@ -1241,7 +1250,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:H4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1262,9 +1271,15 @@
       <c r="F1" t="str">
         <v>permissions</v>
       </c>
+      <c r="G1" t="str">
+        <v>modifiedBy</v>
+      </c>
+      <c r="H1" t="str">
+        <v>modifiedAt</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" t="str">
         <v>1</v>
       </c>
       <c r="B2" t="str">
@@ -1279,9 +1294,15 @@
       <c r="E2" t="str">
         <v>admin</v>
       </c>
+      <c r="G2" t="str">
+        <v>admin</v>
+      </c>
+      <c r="H2" t="str">
+        <v>2025-04-17T12:17:29.351Z</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3">
+      <c r="A3" t="str">
         <v>2</v>
       </c>
       <c r="B3" t="str">
@@ -1296,9 +1317,15 @@
       <c r="E3" t="str">
         <v>user</v>
       </c>
+      <c r="G3" t="str">
+        <v>admin</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2025-04-17T12:18:04.052Z</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4">
+      <c r="A4" t="str">
         <v>3</v>
       </c>
       <c r="B4" t="str">
@@ -1313,10 +1340,16 @@
       <c r="E4" t="str">
         <v>viewer</v>
       </c>
+      <c r="G4" t="str">
+        <v>admin</v>
+      </c>
+      <c r="H4" t="str">
+        <v>2025-04-17T12:18:12.491Z</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>